<commit_message>
update info about processing included in nwb packaging
</commit_message>
<xml_diff>
--- a/code/data_management/meta_data_processing_updated.xlsx
+++ b/code/data_management/meta_data_processing_updated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zhixi\Documents\GitHub\aind-beh-ephys-analysis\code\data_management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D444AE7-BD3D-4E2E-B541-8C4CD419FA91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{552EF19F-8779-4BAF-8CF4-139F1E100C18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="5970" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sessions" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="104">
   <si>
     <t>name</t>
   </si>
@@ -335,6 +335,9 @@
   </si>
   <si>
     <t>dd05a569fae78c78add73d164df8554075cb0c15</t>
+  </si>
+  <si>
+    <t>included in nwb</t>
   </si>
 </sst>
 </file>
@@ -804,18 +807,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="57.33203125" customWidth="1"/>
-    <col min="2" max="2" width="63.75" customWidth="1"/>
+    <col min="2" max="2" width="140.75" customWidth="1"/>
     <col min="3" max="3" width="35.1640625" customWidth="1"/>
     <col min="4" max="4" width="23.25" style="8" customWidth="1"/>
     <col min="5" max="5" width="44" customWidth="1"/>
     <col min="6" max="6" width="40.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:6" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -831,8 +834,11 @@
       <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" s="1" customFormat="1" ht="50" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="F1" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="1" customFormat="1" ht="50" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -846,8 +852,11 @@
       <c r="E2" s="5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="F2" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="9" t="s">
         <v>9</v>
       </c>
@@ -861,8 +870,11 @@
       <c r="E3" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="F3" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
@@ -878,8 +890,11 @@
       <c r="E4" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="F4" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="4" t="s">
         <v>16</v>
       </c>
@@ -893,8 +908,11 @@
       <c r="E5" s="5" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="F5" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A6" s="4" t="s">
         <v>19</v>
       </c>
@@ -908,8 +926,11 @@
       <c r="E6" s="5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="F6" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A7" s="4" t="s">
         <v>22</v>
       </c>
@@ -923,8 +944,11 @@
       <c r="E7" s="5" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="F7" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A8" s="4" t="s">
         <v>25</v>
       </c>
@@ -938,8 +962,11 @@
       <c r="E8" s="5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="F8" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A9" s="4" t="s">
         <v>28</v>
       </c>
@@ -953,8 +980,11 @@
       <c r="E9" s="5" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="F9" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A10" s="4" t="s">
         <v>31</v>
       </c>
@@ -968,8 +998,11 @@
       <c r="E10" s="5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="F10" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="1" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="5" t="s">
         <v>34</v>
       </c>
@@ -983,8 +1016,11 @@
       <c r="E11" s="5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="F11" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="50" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="5" t="s">
         <v>37</v>
       </c>
@@ -998,8 +1034,11 @@
       <c r="E12" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="F12" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="50" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="9" t="s">
         <v>40</v>
       </c>
@@ -1012,8 +1051,11 @@
       <c r="E13" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F13" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="50" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A14" s="9" t="s">
         <v>43</v>
       </c>
@@ -1026,8 +1068,11 @@
       <c r="E14" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" ht="23.65" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F14" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="23.65" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A15" s="9" t="s">
         <v>46</v>
       </c>
@@ -1040,8 +1085,11 @@
       <c r="E15" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" ht="23.65" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F15" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="23.65" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A16" s="9" t="s">
         <v>49</v>
       </c>
@@ -1054,8 +1102,11 @@
       <c r="E16" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="47.15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F16" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A17" s="9" t="s">
         <v>52</v>
       </c>
@@ -1068,8 +1119,11 @@
       <c r="E17" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" ht="23.65" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F17" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="23.65" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A18" s="9" t="s">
         <v>55</v>
       </c>
@@ -1082,8 +1136,11 @@
       <c r="E18" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" ht="23.65" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F18" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="23.65" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A19" s="9" t="s">
         <v>58</v>
       </c>
@@ -1096,8 +1153,11 @@
       <c r="E19" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" ht="23.65" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F19" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="23.65" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A20" s="9" t="s">
         <v>61</v>
       </c>
@@ -1110,8 +1170,11 @@
       <c r="E20" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" ht="23.65" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F20" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="23.65" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A21" s="9" t="s">
         <v>64</v>
       </c>
@@ -1123,6 +1186,9 @@
       </c>
       <c r="E21" t="s">
         <v>66</v>
+      </c>
+      <c r="F21" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1135,7 +1201,7 @@
     <hyperlink ref="D13" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
 

</xml_diff>